<commit_message>
Feat : update interface dan notification
</commit_message>
<xml_diff>
--- a/jadwal_rit_whiteboard.xlsx
+++ b/jadwal_rit_whiteboard.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Tower Control\Mobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{318FDA1C-A243-4879-A712-2F4EB120B401}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BA66729-67A4-4966-AFF8-EFA3FC95F615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="84">
   <si>
     <t>id seller</t>
   </si>
@@ -274,6 +274,9 @@
   </si>
   <si>
     <t>id gudang 3 → id gudang 2 id → drop point 3</t>
+  </si>
+  <si>
+    <t>id drop point 3 → id gudang 2  → id drop point 3</t>
   </si>
 </sst>
 </file>
@@ -1054,7 +1057,7 @@
         <v>9</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>39</v>

</xml_diff>